<commit_message>
Preserve completed operational workspace and release evidence
</commit_message>
<xml_diff>
--- a/outputs/01a128c4-1c8c-71b0-819c-29eaae5a311f/PortCityFC_Analytics_Companion.xlsx
+++ b/outputs/01a128c4-1c8c-71b0-819c-29eaae5a311f/PortCityFC_Analytics_Companion.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ownership Snapshot" sheetId="1" r:id="R6ecf846edccf48c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Cash" sheetId="2" r:id="Re17c789d14b54ef3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income &amp; Expense" sheetId="3" r:id="R6a4c4de650e14ea1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operating Assumptions" sheetId="4" r:id="Rd61850e3001442a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="5" r:id="R6c4a7b476be6484e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Star Schema" sheetId="6" r:id="Ra0c37eec3e324461"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="7" r:id="R68d98f901a2f45ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="8" r:id="R7b816d4264e946b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ownership Snapshot" sheetId="1" r:id="R2eb9d2821e3e447a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Cash" sheetId="2" r:id="Rbcd65b300b844461"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income &amp; Expense" sheetId="3" r:id="R3d13abda4b924c6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operating Assumptions" sheetId="4" r:id="Rf6724080dae74738"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="5" r:id="R86d1b039cced4167"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Star Schema" sheetId="6" r:id="R0ba4740705504120"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="7" r:id="Rcb29969f498e4bbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="8" r:id="Rbf2ee6dd0b8b4c8e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,14 +20,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="$#,##0;[Red]-$#,##0"/>
     <x:numFmt numFmtId="201" formatCode="$#,##0"/>
     <x:numFmt numFmtId="202" formatCode="0.0%"/>
     <x:numFmt numFmtId="203" formatCode="0.0"/>
     <x:numFmt numFmtId="204" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="205" formatCode="$#,##0;($#,##0);&quot;–&quot;"/>
   </x:numFmts>
-  <x:fonts count="14">
+  <x:fonts count="20">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -106,8 +107,41 @@
       <x:color rgb="FF7C4A03"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF0000FF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="20"/>
+      <x:color rgb="FF142033"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF008000"/>
+      <x:name val="Aptos"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -147,6 +181,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF7E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B2942"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B2942"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B2942"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -304,7 +353,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="210">
+  <x:cellXfs count="245">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -699,10 +748,183 @@
     <x:xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="16" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="16" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="17" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="18" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="18" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="19" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
+  <x:dxfs count="6">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB91C1C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB91C1C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB91C1C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB91C1C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB91C1C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FFB91C1C"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFEE2E2"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+  </x:dxfs>
 </x:styleSheet>
 </file>
 
@@ -723,7 +945,7 @@
                 <a:ea typeface="Aptos"/>
                 <a:cs typeface="Aptos"/>
               </a:rPr>
-              <a:t>Cash movement by month</a:t>
+              <a:t>Monthly cash receipts &amp; payments · FY25</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -937,7 +1159,7 @@
                 <a:ea typeface="Aptos"/>
                 <a:cs typeface="Aptos"/>
               </a:rPr>
-              <a:t>Largest modeled income categories</a:t>
+              <a:t>FY25 synthetic income categories</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1105,7 +1327,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re847c2f1c1894ce9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R40e68b63d07741e0"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1135,7 +1357,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R78639e3b8a254641"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R62bd76a2cf684084"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1527,7 +1749,7 @@
       <x:c r="G5" s="66"/>
       <x:c r="H5" s="200"/>
       <x:c r="I5" s="64" t="str">
-        <x:v>NET CASH</x:v>
+        <x:v>FY25 NET CASH CHANGE</x:v>
       </x:c>
       <x:c r="J5" s="65"/>
       <x:c r="K5" s="66"/>
@@ -1546,32 +1768,32 @@
       <x:c r="V5" s="200"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="86" t="n">
+      <x:c r="A6" s="220" t="n">
         <x:f>'Monthly Cash'!B18</x:f>
         <x:v>67500</x:v>
       </x:c>
-      <x:c r="B6" s="87"/>
-      <x:c r="C6" s="88"/>
+      <x:c r="B6" s="221"/>
+      <x:c r="C6" s="222"/>
       <x:c r="D6" s="200"/>
-      <x:c r="E6" s="113" t="n">
+      <x:c r="E6" s="220" t="n">
         <x:f>'Monthly Cash'!C18</x:f>
         <x:v>63700</x:v>
       </x:c>
-      <x:c r="F6" s="114"/>
-      <x:c r="G6" s="115"/>
+      <x:c r="F6" s="221"/>
+      <x:c r="G6" s="222"/>
       <x:c r="H6" s="200"/>
-      <x:c r="I6" s="140" t="n">
+      <x:c r="I6" s="220" t="n">
         <x:f>'Monthly Cash'!D18</x:f>
         <x:v>3800</x:v>
       </x:c>
-      <x:c r="J6" s="141"/>
-      <x:c r="K6" s="142"/>
+      <x:c r="J6" s="221"/>
+      <x:c r="K6" s="222"/>
       <x:c r="L6" s="200"/>
-      <x:c r="M6" s="162" t="n">
-        <x:f>I6/A6</x:f>
+      <x:c r="M6" s="229" t="n">
+        <x:f>IF(A6=0,"n.a.",I6/A6)</x:f>
         <x:v>0.056296296296296296</x:v>
       </x:c>
-      <x:c r="N6" s="163"/>
+      <x:c r="N6" s="230"/>
       <x:c r="O6" s="200"/>
       <x:c r="P6" s="200"/>
       <x:c r="Q6" s="200"/>
@@ -1582,20 +1804,20 @@
       <x:c r="V6" s="200"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="89"/>
-      <x:c r="B7" s="90"/>
-      <x:c r="C7" s="91"/>
+      <x:c r="A7" s="223"/>
+      <x:c r="B7" s="224"/>
+      <x:c r="C7" s="225"/>
       <x:c r="D7" s="200"/>
-      <x:c r="E7" s="116"/>
-      <x:c r="F7" s="117"/>
-      <x:c r="G7" s="118"/>
+      <x:c r="E7" s="223"/>
+      <x:c r="F7" s="224"/>
+      <x:c r="G7" s="225"/>
       <x:c r="H7" s="200"/>
-      <x:c r="I7" s="143"/>
-      <x:c r="J7" s="144"/>
-      <x:c r="K7" s="145"/>
+      <x:c r="I7" s="223"/>
+      <x:c r="J7" s="224"/>
+      <x:c r="K7" s="225"/>
       <x:c r="L7" s="200"/>
-      <x:c r="M7" s="164"/>
-      <x:c r="N7" s="165"/>
+      <x:c r="M7" s="231"/>
+      <x:c r="N7" s="232"/>
       <x:c r="O7" s="200"/>
       <x:c r="P7" s="200"/>
       <x:c r="Q7" s="200"/>
@@ -1606,20 +1828,20 @@
       <x:c r="V7" s="200"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="92"/>
-      <x:c r="B8" s="93"/>
-      <x:c r="C8" s="94"/>
+      <x:c r="A8" s="226"/>
+      <x:c r="B8" s="227"/>
+      <x:c r="C8" s="228"/>
       <x:c r="D8" s="200"/>
-      <x:c r="E8" s="119"/>
-      <x:c r="F8" s="120"/>
-      <x:c r="G8" s="121"/>
+      <x:c r="E8" s="226"/>
+      <x:c r="F8" s="227"/>
+      <x:c r="G8" s="228"/>
       <x:c r="H8" s="200"/>
-      <x:c r="I8" s="146"/>
-      <x:c r="J8" s="147"/>
-      <x:c r="K8" s="148"/>
+      <x:c r="I8" s="226"/>
+      <x:c r="J8" s="227"/>
+      <x:c r="K8" s="228"/>
       <x:c r="L8" s="200"/>
-      <x:c r="M8" s="166"/>
-      <x:c r="N8" s="167"/>
+      <x:c r="M8" s="233"/>
+      <x:c r="N8" s="234"/>
       <x:c r="O8" s="200"/>
       <x:c r="P8" s="200"/>
       <x:c r="Q8" s="200"/>
@@ -2063,7 +2285,7 @@
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="11" t="str">
-        <x:v>OWNER DECISIONS</x:v>
+        <x:v>SUGGESTED REVIEW ACTIONS · NOT APPROVED CLUB DECISIONS</x:v>
       </x:c>
       <x:c r="B27" s="11"/>
       <x:c r="C27" s="11"/>
@@ -2127,18 +2349,18 @@
       <x:c r="C29" s="171"/>
       <x:c r="D29" s="171"/>
       <x:c r="E29" s="171" t="str">
-        <x:v>Commercial lead • 30 days</x:v>
+        <x:v>Commercial lead · proposed</x:v>
       </x:c>
       <x:c r="F29" s="171"/>
       <x:c r="G29" s="171"/>
       <x:c r="H29" s="171" t="str">
-        <x:v>Synthetic mix • pipeline coverage</x:v>
+        <x:v>Synthetic concentration only</x:v>
       </x:c>
       <x:c r="I29" s="171"/>
       <x:c r="J29" s="171"/>
       <x:c r="K29" s="171"/>
       <x:c r="L29" s="171" t="str">
-        <x:v>OPEN • monthly</x:v>
+        <x:v>PROPOSED · unassigned</x:v>
       </x:c>
       <x:c r="M29" s="171"/>
       <x:c r="N29" s="171"/>
@@ -2159,18 +2381,18 @@
       <x:c r="C30" s="171"/>
       <x:c r="D30" s="171"/>
       <x:c r="E30" s="171" t="str">
-        <x:v>Operations lead • pre-season</x:v>
+        <x:v>Operations lead · proposed</x:v>
       </x:c>
       <x:c r="F30" s="171"/>
       <x:c r="G30" s="171"/>
       <x:c r="H30" s="171" t="str">
-        <x:v>Modeled cost • contracted ceiling</x:v>
+        <x:v>Do not add commitments to ledger</x:v>
       </x:c>
       <x:c r="I30" s="171"/>
       <x:c r="J30" s="171"/>
       <x:c r="K30" s="171"/>
       <x:c r="L30" s="171" t="str">
-        <x:v>OPEN • weekly</x:v>
+        <x:v>PROPOSED · unassigned</x:v>
       </x:c>
       <x:c r="M30" s="171"/>
       <x:c r="N30" s="171"/>
@@ -2191,18 +2413,18 @@
       <x:c r="C31" s="171"/>
       <x:c r="D31" s="171"/>
       <x:c r="E31" s="171" t="str">
-        <x:v>Executive sponsor • immediate</x:v>
+        <x:v>Executive sponsor · proposed</x:v>
       </x:c>
       <x:c r="F31" s="171"/>
       <x:c r="G31" s="171"/>
       <x:c r="H31" s="171" t="str">
-        <x:v>Audited workflow • named approver</x:v>
+        <x:v>Versioned workflow; club review needed</x:v>
       </x:c>
       <x:c r="I31" s="171"/>
       <x:c r="J31" s="171"/>
       <x:c r="K31" s="171"/>
       <x:c r="L31" s="171" t="str">
-        <x:v>READY • quarterly</x:v>
+        <x:v>PROPOSED · unassigned</x:v>
       </x:c>
       <x:c r="M31" s="171"/>
       <x:c r="N31" s="171"/>
@@ -2223,18 +2445,18 @@
       <x:c r="C32" s="171"/>
       <x:c r="D32" s="171"/>
       <x:c r="E32" s="171" t="str">
-        <x:v>Analytics lead • next fixture</x:v>
+        <x:v>Analytics lead · proposed</x:v>
       </x:c>
       <x:c r="F32" s="171"/>
       <x:c r="G32" s="171"/>
       <x:c r="H32" s="171" t="str">
-        <x:v>Sanitized input • ticket scan source</x:v>
+        <x:v>Sample ≠ complete season</x:v>
       </x:c>
       <x:c r="I32" s="171"/>
       <x:c r="J32" s="171"/>
       <x:c r="K32" s="171"/>
       <x:c r="L32" s="171" t="str">
-        <x:v>OPEN • post-match</x:v>
+        <x:v>PROPOSED · unassigned</x:v>
       </x:c>
       <x:c r="M32" s="171"/>
       <x:c r="N32" s="171"/>
@@ -2299,7 +2521,7 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="191" t="str">
-        <x:v>All public figures are synthetic or sanitized assumptions. The reproducible pipeline reconciles every displayed finance total; private staff contacts, transaction rows, payees, source filenames, and interview attribution are excluded.</x:v>
+        <x:v>Source reference 2026-10-12. Synthetic portfolio model, not certified PCFC accounts. Net cash change is not bank balance, profit or runway. FY24 has annual totals only. Private records and public demonstration data remain separate.</x:v>
       </x:c>
       <x:c r="B35" s="192"/>
       <x:c r="C35" s="192"/>
@@ -2395,21 +2617,23 @@
       <x:c r="U38" s="200"/>
       <x:c r="V38" s="200"/>
     </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="200"/>
-      <x:c r="B39" s="200"/>
-      <x:c r="C39" s="200"/>
-      <x:c r="D39" s="200"/>
-      <x:c r="E39" s="200"/>
-      <x:c r="F39" s="200"/>
-      <x:c r="G39" s="200"/>
-      <x:c r="H39" s="200"/>
-      <x:c r="I39" s="200"/>
-      <x:c r="J39" s="200"/>
-      <x:c r="K39" s="200"/>
-      <x:c r="L39" s="200"/>
-      <x:c r="M39" s="200"/>
-      <x:c r="N39" s="200"/>
+    <x:row r="39" ht="24" customHeight="1">
+      <x:c r="A39" s="244" t="str">
+        <x:v>ANNUAL COMPARISON · USD · SYNTHETIC</x:v>
+      </x:c>
+      <x:c r="B39" s="244"/>
+      <x:c r="C39" s="244"/>
+      <x:c r="D39" s="244"/>
+      <x:c r="E39" s="244"/>
+      <x:c r="F39" s="244"/>
+      <x:c r="G39" s="244"/>
+      <x:c r="H39" s="244"/>
+      <x:c r="I39" s="244"/>
+      <x:c r="J39" s="244"/>
+      <x:c r="K39" s="244"/>
+      <x:c r="L39" s="244"/>
+      <x:c r="M39" s="244"/>
+      <x:c r="N39" s="244"/>
       <x:c r="O39" s="200"/>
       <x:c r="P39" s="200"/>
       <x:c r="Q39" s="200"/>
@@ -2419,20 +2643,28 @@
       <x:c r="U39" s="200"/>
       <x:c r="V39" s="200"/>
     </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="200"/>
+    <x:row r="40" ht="24" customHeight="1">
+      <x:c r="A40" s="200" t="str">
+        <x:v>Period</x:v>
+      </x:c>
       <x:c r="B40" s="200"/>
       <x:c r="C40" s="200"/>
       <x:c r="D40" s="200"/>
-      <x:c r="E40" s="200"/>
+      <x:c r="E40" s="200" t="str">
+        <x:v>Inflow</x:v>
+      </x:c>
       <x:c r="F40" s="200"/>
       <x:c r="G40" s="200"/>
       <x:c r="H40" s="200"/>
-      <x:c r="I40" s="200"/>
+      <x:c r="I40" s="200" t="str">
+        <x:v>Outflow</x:v>
+      </x:c>
       <x:c r="J40" s="200"/>
       <x:c r="K40" s="200"/>
       <x:c r="L40" s="200"/>
-      <x:c r="M40" s="200"/>
+      <x:c r="M40" s="200" t="str">
+        <x:v>Net cash change</x:v>
+      </x:c>
       <x:c r="N40" s="200"/>
       <x:c r="O40" s="200"/>
       <x:c r="P40" s="200"/>
@@ -2443,21 +2675,30 @@
       <x:c r="U40" s="200"/>
       <x:c r="V40" s="200"/>
     </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="200"/>
-      <x:c r="B41" s="200"/>
-      <x:c r="C41" s="200"/>
-      <x:c r="D41" s="200"/>
-      <x:c r="E41" s="200"/>
-      <x:c r="F41" s="200"/>
-      <x:c r="G41" s="200"/>
-      <x:c r="H41" s="200"/>
-      <x:c r="I41" s="200"/>
-      <x:c r="J41" s="200"/>
-      <x:c r="K41" s="200"/>
-      <x:c r="L41" s="200"/>
-      <x:c r="M41" s="200"/>
-      <x:c r="N41" s="200"/>
+    <x:row r="41" ht="24" customHeight="1">
+      <x:c r="A41" s="200" t="str">
+        <x:v>FY24</x:v>
+      </x:c>
+      <x:c r="B41" s="239"/>
+      <x:c r="C41" s="239"/>
+      <x:c r="D41" s="239"/>
+      <x:c r="E41" s="239" t="n">
+        <x:v>63200</x:v>
+      </x:c>
+      <x:c r="F41" s="239"/>
+      <x:c r="G41" s="239"/>
+      <x:c r="H41" s="239"/>
+      <x:c r="I41" s="239" t="n">
+        <x:v>60950</x:v>
+      </x:c>
+      <x:c r="J41" s="239"/>
+      <x:c r="K41" s="239"/>
+      <x:c r="L41" s="239"/>
+      <x:c r="M41" s="239" t="n">
+        <x:f>E41-I41</x:f>
+        <x:v>2250</x:v>
+      </x:c>
+      <x:c r="N41" s="239"/>
       <x:c r="O41" s="200"/>
       <x:c r="P41" s="200"/>
       <x:c r="Q41" s="200"/>
@@ -2467,21 +2708,30 @@
       <x:c r="U41" s="200"/>
       <x:c r="V41" s="200"/>
     </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="200"/>
-      <x:c r="B42" s="200"/>
-      <x:c r="C42" s="200"/>
-      <x:c r="D42" s="200"/>
-      <x:c r="E42" s="200"/>
-      <x:c r="F42" s="200"/>
-      <x:c r="G42" s="200"/>
-      <x:c r="H42" s="200"/>
-      <x:c r="I42" s="200"/>
-      <x:c r="J42" s="200"/>
-      <x:c r="K42" s="200"/>
-      <x:c r="L42" s="200"/>
-      <x:c r="M42" s="200"/>
-      <x:c r="N42" s="200"/>
+    <x:row r="42" ht="24" customHeight="1">
+      <x:c r="A42" s="200" t="str">
+        <x:v>FY25</x:v>
+      </x:c>
+      <x:c r="B42" s="239"/>
+      <x:c r="C42" s="239"/>
+      <x:c r="D42" s="239"/>
+      <x:c r="E42" s="239" t="n">
+        <x:v>67500</x:v>
+      </x:c>
+      <x:c r="F42" s="239"/>
+      <x:c r="G42" s="239"/>
+      <x:c r="H42" s="239"/>
+      <x:c r="I42" s="239" t="n">
+        <x:v>63700</x:v>
+      </x:c>
+      <x:c r="J42" s="239"/>
+      <x:c r="K42" s="239"/>
+      <x:c r="L42" s="239"/>
+      <x:c r="M42" s="239" t="n">
+        <x:f>E42-I42</x:f>
+        <x:v>3800</x:v>
+      </x:c>
+      <x:c r="N42" s="239"/>
       <x:c r="O42" s="200"/>
       <x:c r="P42" s="200"/>
       <x:c r="Q42" s="200"/>
@@ -2526,9 +2776,22 @@
     <x:mergeCell ref="L32:N32"/>
     <x:mergeCell ref="A34:N34"/>
     <x:mergeCell ref="A35:N37"/>
+    <x:mergeCell ref="A39:N39"/>
+    <x:mergeCell ref="A40:C40"/>
+    <x:mergeCell ref="E40:G40"/>
+    <x:mergeCell ref="I40:K40"/>
+    <x:mergeCell ref="M40:N40"/>
+    <x:mergeCell ref="A41:C41"/>
+    <x:mergeCell ref="E41:G41"/>
+    <x:mergeCell ref="I41:K41"/>
+    <x:mergeCell ref="M41:N41"/>
+    <x:mergeCell ref="A42:C42"/>
+    <x:mergeCell ref="E42:G42"/>
+    <x:mergeCell ref="I42:K42"/>
+    <x:mergeCell ref="M42:N42"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc47cee2f1094eb2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92e68df9d04f48fa"/>
 </x:worksheet>
 </file>
 
@@ -2546,7 +2809,7 @@
   <x:sheetData>
     <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>Monthly Cash Movement</x:v>
+        <x:v>Monthly Cash Receipts &amp; Payments</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -2604,17 +2867,17 @@
       <x:c r="A6" s="201" t="str">
         <x:v>Jan</x:v>
       </x:c>
-      <x:c r="B6" s="202" t="n">
+      <x:c r="B6" s="213" t="n">
         <x:v>6000</x:v>
       </x:c>
-      <x:c r="C6" s="202" t="n">
+      <x:c r="C6" s="213" t="n">
         <x:v>2500</x:v>
       </x:c>
-      <x:c r="D6" s="202" t="n">
+      <x:c r="D6" s="214" t="n">
         <x:f>B6-C6</x:f>
         <x:v>3500</x:v>
       </x:c>
-      <x:c r="E6" s="202" t="n">
+      <x:c r="E6" s="214" t="n">
         <x:f>D6</x:f>
         <x:v>3500</x:v>
       </x:c>
@@ -2626,17 +2889,17 @@
       <x:c r="A7" s="201" t="str">
         <x:v>Feb</x:v>
       </x:c>
-      <x:c r="B7" s="202" t="n">
+      <x:c r="B7" s="213" t="n">
         <x:v>5000</x:v>
       </x:c>
-      <x:c r="C7" s="202" t="n">
+      <x:c r="C7" s="213" t="n">
         <x:v>3200</x:v>
       </x:c>
-      <x:c r="D7" s="202" t="n">
+      <x:c r="D7" s="214" t="n">
         <x:f>B7-C7</x:f>
         <x:v>1800</x:v>
       </x:c>
-      <x:c r="E7" s="202" t="n">
+      <x:c r="E7" s="214" t="n">
         <x:f>E6+D7</x:f>
         <x:v>5300</x:v>
       </x:c>
@@ -2648,17 +2911,17 @@
       <x:c r="A8" s="201" t="str">
         <x:v>Mar</x:v>
       </x:c>
-      <x:c r="B8" s="202" t="n">
+      <x:c r="B8" s="213" t="n">
         <x:v>7500</x:v>
       </x:c>
-      <x:c r="C8" s="202" t="n">
+      <x:c r="C8" s="213" t="n">
         <x:v>3800</x:v>
       </x:c>
-      <x:c r="D8" s="202" t="n">
+      <x:c r="D8" s="214" t="n">
         <x:f>B8-C8</x:f>
         <x:v>3700</x:v>
       </x:c>
-      <x:c r="E8" s="202" t="n">
+      <x:c r="E8" s="214" t="n">
         <x:f>E7+D8</x:f>
         <x:v>9000</x:v>
       </x:c>
@@ -2670,17 +2933,17 @@
       <x:c r="A9" s="201" t="str">
         <x:v>Apr</x:v>
       </x:c>
-      <x:c r="B9" s="202" t="n">
+      <x:c r="B9" s="213" t="n">
         <x:v>8000</x:v>
       </x:c>
-      <x:c r="C9" s="202" t="n">
+      <x:c r="C9" s="213" t="n">
         <x:v>4200</x:v>
       </x:c>
-      <x:c r="D9" s="202" t="n">
+      <x:c r="D9" s="214" t="n">
         <x:f>B9-C9</x:f>
         <x:v>3800</x:v>
       </x:c>
-      <x:c r="E9" s="202" t="n">
+      <x:c r="E9" s="214" t="n">
         <x:f>E8+D9</x:f>
         <x:v>12800</x:v>
       </x:c>
@@ -2692,17 +2955,17 @@
       <x:c r="A10" s="201" t="str">
         <x:v>May</x:v>
       </x:c>
-      <x:c r="B10" s="202" t="n">
+      <x:c r="B10" s="213" t="n">
         <x:v>7000</x:v>
       </x:c>
-      <x:c r="C10" s="202" t="n">
+      <x:c r="C10" s="213" t="n">
         <x:v>5200</x:v>
       </x:c>
-      <x:c r="D10" s="202" t="n">
+      <x:c r="D10" s="214" t="n">
         <x:f>B10-C10</x:f>
         <x:v>1800</x:v>
       </x:c>
-      <x:c r="E10" s="202" t="n">
+      <x:c r="E10" s="214" t="n">
         <x:f>E9+D10</x:f>
         <x:v>14600</x:v>
       </x:c>
@@ -2714,17 +2977,17 @@
       <x:c r="A11" s="201" t="str">
         <x:v>Jun</x:v>
       </x:c>
-      <x:c r="B11" s="202" t="n">
+      <x:c r="B11" s="213" t="n">
         <x:v>6000</x:v>
       </x:c>
-      <x:c r="C11" s="202" t="n">
+      <x:c r="C11" s="213" t="n">
         <x:v>6100</x:v>
       </x:c>
-      <x:c r="D11" s="202" t="n">
+      <x:c r="D11" s="214" t="n">
         <x:f>B11-C11</x:f>
         <x:v>-100</x:v>
       </x:c>
-      <x:c r="E11" s="202" t="n">
+      <x:c r="E11" s="214" t="n">
         <x:f>E10+D11</x:f>
         <x:v>14500</x:v>
       </x:c>
@@ -2736,17 +2999,17 @@
       <x:c r="A12" s="201" t="str">
         <x:v>Jul</x:v>
       </x:c>
-      <x:c r="B12" s="202" t="n">
+      <x:c r="B12" s="213" t="n">
         <x:v>6500</x:v>
       </x:c>
-      <x:c r="C12" s="202" t="n">
+      <x:c r="C12" s="213" t="n">
         <x:v>7400</x:v>
       </x:c>
-      <x:c r="D12" s="202" t="n">
+      <x:c r="D12" s="214" t="n">
         <x:f>B12-C12</x:f>
         <x:v>-900</x:v>
       </x:c>
-      <x:c r="E12" s="202" t="n">
+      <x:c r="E12" s="214" t="n">
         <x:f>E11+D12</x:f>
         <x:v>13600</x:v>
       </x:c>
@@ -2758,17 +3021,17 @@
       <x:c r="A13" s="201" t="str">
         <x:v>Aug</x:v>
       </x:c>
-      <x:c r="B13" s="202" t="n">
+      <x:c r="B13" s="213" t="n">
         <x:v>7500</x:v>
       </x:c>
-      <x:c r="C13" s="202" t="n">
+      <x:c r="C13" s="213" t="n">
         <x:v>8200</x:v>
       </x:c>
-      <x:c r="D13" s="202" t="n">
+      <x:c r="D13" s="214" t="n">
         <x:f>B13-C13</x:f>
         <x:v>-700</x:v>
       </x:c>
-      <x:c r="E13" s="202" t="n">
+      <x:c r="E13" s="214" t="n">
         <x:f>E12+D13</x:f>
         <x:v>12900</x:v>
       </x:c>
@@ -2780,17 +3043,17 @@
       <x:c r="A14" s="201" t="str">
         <x:v>Sep</x:v>
       </x:c>
-      <x:c r="B14" s="202" t="n">
+      <x:c r="B14" s="213" t="n">
         <x:v>5000</x:v>
       </x:c>
-      <x:c r="C14" s="202" t="n">
+      <x:c r="C14" s="213" t="n">
         <x:v>7600</x:v>
       </x:c>
-      <x:c r="D14" s="202" t="n">
+      <x:c r="D14" s="214" t="n">
         <x:f>B14-C14</x:f>
         <x:v>-2600</x:v>
       </x:c>
-      <x:c r="E14" s="202" t="n">
+      <x:c r="E14" s="214" t="n">
         <x:f>E13+D14</x:f>
         <x:v>10300</x:v>
       </x:c>
@@ -2802,17 +3065,17 @@
       <x:c r="A15" s="201" t="str">
         <x:v>Oct</x:v>
       </x:c>
-      <x:c r="B15" s="202" t="n">
+      <x:c r="B15" s="213" t="n">
         <x:v>4500</x:v>
       </x:c>
-      <x:c r="C15" s="202" t="n">
+      <x:c r="C15" s="213" t="n">
         <x:v>6000</x:v>
       </x:c>
-      <x:c r="D15" s="202" t="n">
+      <x:c r="D15" s="214" t="n">
         <x:f>B15-C15</x:f>
         <x:v>-1500</x:v>
       </x:c>
-      <x:c r="E15" s="202" t="n">
+      <x:c r="E15" s="214" t="n">
         <x:f>E14+D15</x:f>
         <x:v>8800</x:v>
       </x:c>
@@ -2824,17 +3087,17 @@
       <x:c r="A16" s="201" t="str">
         <x:v>Nov</x:v>
       </x:c>
-      <x:c r="B16" s="202" t="n">
+      <x:c r="B16" s="213" t="n">
         <x:v>2500</x:v>
       </x:c>
-      <x:c r="C16" s="202" t="n">
+      <x:c r="C16" s="213" t="n">
         <x:v>5100</x:v>
       </x:c>
-      <x:c r="D16" s="202" t="n">
+      <x:c r="D16" s="214" t="n">
         <x:f>B16-C16</x:f>
         <x:v>-2600</x:v>
       </x:c>
-      <x:c r="E16" s="202" t="n">
+      <x:c r="E16" s="214" t="n">
         <x:f>E15+D16</x:f>
         <x:v>6200</x:v>
       </x:c>
@@ -2846,17 +3109,17 @@
       <x:c r="A17" s="201" t="str">
         <x:v>Dec</x:v>
       </x:c>
-      <x:c r="B17" s="202" t="n">
+      <x:c r="B17" s="213" t="n">
         <x:v>2000</x:v>
       </x:c>
-      <x:c r="C17" s="202" t="n">
+      <x:c r="C17" s="213" t="n">
         <x:v>4400</x:v>
       </x:c>
-      <x:c r="D17" s="202" t="n">
+      <x:c r="D17" s="214" t="n">
         <x:f>B17-C17</x:f>
         <x:v>-2400</x:v>
       </x:c>
-      <x:c r="E17" s="202" t="n">
+      <x:c r="E17" s="214" t="n">
         <x:f>E16+D17</x:f>
         <x:v>3800</x:v>
       </x:c>
@@ -2868,19 +3131,19 @@
       <x:c r="A18" s="203" t="str">
         <x:v>Control total</x:v>
       </x:c>
-      <x:c r="B18" s="204" t="n">
+      <x:c r="B18" s="215" t="n">
         <x:f>SUM(B6:B17)</x:f>
         <x:v>67500</x:v>
       </x:c>
-      <x:c r="C18" s="204" t="n">
+      <x:c r="C18" s="215" t="n">
         <x:f>SUM(C6:C17)</x:f>
         <x:v>63700</x:v>
       </x:c>
-      <x:c r="D18" s="204" t="n">
+      <x:c r="D18" s="216" t="n">
         <x:f>SUM(D6:D17)</x:f>
         <x:v>3800</x:v>
       </x:c>
-      <x:c r="E18" s="204" t="n">
+      <x:c r="E18" s="216" t="n">
         <x:f>E17</x:f>
         <x:v>3800</x:v>
       </x:c>
@@ -2909,7 +3172,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R36fbf6215b104a32"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R227ac946ec0b4004"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2981,11 +3244,11 @@
       <x:c r="B6" s="201" t="str">
         <x:v>Inflow</x:v>
       </x:c>
-      <x:c r="C6" s="205" t="n">
+      <x:c r="C6" s="217" t="n">
         <x:v>38000</x:v>
       </x:c>
-      <x:c r="D6" s="206" t="n">
-        <x:f>C6/SUMIF($B$6:$B$19,B6,$C$6:$C$19)</x:f>
+      <x:c r="D6" s="218" t="n">
+        <x:f>IF(SUMIF($B$6:$B$19,B6,$C$6:$C$19)=0,"n.a.",C6/SUMIF($B$6:$B$19,B6,$C$6:$C$19))</x:f>
         <x:v>0.562962962962963</x:v>
       </x:c>
       <x:c r="E6" s="201" t="str">
@@ -2999,11 +3262,11 @@
       <x:c r="B7" s="201" t="str">
         <x:v>Inflow</x:v>
       </x:c>
-      <x:c r="C7" s="205" t="n">
+      <x:c r="C7" s="217" t="n">
         <x:v>15400</x:v>
       </x:c>
-      <x:c r="D7" s="206" t="n">
-        <x:f>C7/SUMIF($B$6:$B$19,B7,$C$6:$C$19)</x:f>
+      <x:c r="D7" s="218" t="n">
+        <x:f>IF(SUMIF($B$6:$B$19,B7,$C$6:$C$19)=0,"n.a.",C7/SUMIF($B$6:$B$19,B7,$C$6:$C$19))</x:f>
         <x:v>0.22814814814814816</x:v>
       </x:c>
       <x:c r="E7" s="201" t="str">
@@ -3017,11 +3280,11 @@
       <x:c r="B8" s="201" t="str">
         <x:v>Inflow</x:v>
       </x:c>
-      <x:c r="C8" s="205" t="n">
+      <x:c r="C8" s="217" t="n">
         <x:v>6400</x:v>
       </x:c>
-      <x:c r="D8" s="206" t="n">
-        <x:f>C8/SUMIF($B$6:$B$19,B8,$C$6:$C$19)</x:f>
+      <x:c r="D8" s="218" t="n">
+        <x:f>IF(SUMIF($B$6:$B$19,B8,$C$6:$C$19)=0,"n.a.",C8/SUMIF($B$6:$B$19,B8,$C$6:$C$19))</x:f>
         <x:v>0.09481481481481481</x:v>
       </x:c>
       <x:c r="E8" s="201" t="str">
@@ -3035,11 +3298,11 @@
       <x:c r="B9" s="201" t="str">
         <x:v>Inflow</x:v>
       </x:c>
-      <x:c r="C9" s="205" t="n">
+      <x:c r="C9" s="217" t="n">
         <x:v>4200</x:v>
       </x:c>
-      <x:c r="D9" s="206" t="n">
-        <x:f>C9/SUMIF($B$6:$B$19,B9,$C$6:$C$19)</x:f>
+      <x:c r="D9" s="218" t="n">
+        <x:f>IF(SUMIF($B$6:$B$19,B9,$C$6:$C$19)=0,"n.a.",C9/SUMIF($B$6:$B$19,B9,$C$6:$C$19))</x:f>
         <x:v>0.06222222222222222</x:v>
       </x:c>
       <x:c r="E9" s="201" t="str">
@@ -3053,11 +3316,11 @@
       <x:c r="B10" s="201" t="str">
         <x:v>Inflow</x:v>
       </x:c>
-      <x:c r="C10" s="205" t="n">
+      <x:c r="C10" s="217" t="n">
         <x:v>2100</x:v>
       </x:c>
-      <x:c r="D10" s="206" t="n">
-        <x:f>C10/SUMIF($B$6:$B$19,B10,$C$6:$C$19)</x:f>
+      <x:c r="D10" s="218" t="n">
+        <x:f>IF(SUMIF($B$6:$B$19,B10,$C$6:$C$19)=0,"n.a.",C10/SUMIF($B$6:$B$19,B10,$C$6:$C$19))</x:f>
         <x:v>0.03111111111111111</x:v>
       </x:c>
       <x:c r="E10" s="201" t="str">
@@ -3071,11 +3334,11 @@
       <x:c r="B11" s="201" t="str">
         <x:v>Inflow</x:v>
       </x:c>
-      <x:c r="C11" s="205" t="n">
+      <x:c r="C11" s="217" t="n">
         <x:v>1400</x:v>
       </x:c>
-      <x:c r="D11" s="206" t="n">
-        <x:f>C11/SUMIF($B$6:$B$19,B11,$C$6:$C$19)</x:f>
+      <x:c r="D11" s="218" t="n">
+        <x:f>IF(SUMIF($B$6:$B$19,B11,$C$6:$C$19)=0,"n.a.",C11/SUMIF($B$6:$B$19,B11,$C$6:$C$19))</x:f>
         <x:v>0.02074074074074074</x:v>
       </x:c>
       <x:c r="E11" s="201" t="str">
@@ -3089,11 +3352,11 @@
       <x:c r="B12" s="201" t="str">
         <x:v>Outflow</x:v>
       </x:c>
-      <x:c r="C12" s="205" t="n">
+      <x:c r="C12" s="217" t="n">
         <x:v>14200</x:v>
       </x:c>
-      <x:c r="D12" s="206" t="n">
-        <x:f>C12/SUMIF($B$6:$B$19,B12,$C$6:$C$19)</x:f>
+      <x:c r="D12" s="218" t="n">
+        <x:f>IF(SUMIF($B$6:$B$19,B12,$C$6:$C$19)=0,"n.a.",C12/SUMIF($B$6:$B$19,B12,$C$6:$C$19))</x:f>
         <x:v>0.22291993720565148</x:v>
       </x:c>
       <x:c r="E12" s="201" t="str">
@@ -3107,11 +3370,11 @@
       <x:c r="B13" s="201" t="str">
         <x:v>Outflow</x:v>
       </x:c>
-      <x:c r="C13" s="205" t="n">
+      <x:c r="C13" s="217" t="n">
         <x:v>13600</x:v>
       </x:c>
-      <x:c r="D13" s="206" t="n">
-        <x:f>C13/SUMIF($B$6:$B$19,B13,$C$6:$C$19)</x:f>
+      <x:c r="D13" s="218" t="n">
+        <x:f>IF(SUMIF($B$6:$B$19,B13,$C$6:$C$19)=0,"n.a.",C13/SUMIF($B$6:$B$19,B13,$C$6:$C$19))</x:f>
         <x:v>0.21350078492935637</x:v>
       </x:c>
       <x:c r="E13" s="201" t="str">
@@ -3125,11 +3388,11 @@
       <x:c r="B14" s="201" t="str">
         <x:v>Outflow</x:v>
       </x:c>
-      <x:c r="C14" s="205" t="n">
+      <x:c r="C14" s="217" t="n">
         <x:v>9400</x:v>
       </x:c>
-      <x:c r="D14" s="206" t="n">
-        <x:f>C14/SUMIF($B$6:$B$19,B14,$C$6:$C$19)</x:f>
+      <x:c r="D14" s="218" t="n">
+        <x:f>IF(SUMIF($B$6:$B$19,B14,$C$6:$C$19)=0,"n.a.",C14/SUMIF($B$6:$B$19,B14,$C$6:$C$19))</x:f>
         <x:v>0.14756671899529042</x:v>
       </x:c>
       <x:c r="E14" s="201" t="str">
@@ -3143,11 +3406,11 @@
       <x:c r="B15" s="201" t="str">
         <x:v>Outflow</x:v>
       </x:c>
-      <x:c r="C15" s="205" t="n">
+      <x:c r="C15" s="217" t="n">
         <x:v>8100</x:v>
       </x:c>
-      <x:c r="D15" s="206" t="n">
-        <x:f>C15/SUMIF($B$6:$B$19,B15,$C$6:$C$19)</x:f>
+      <x:c r="D15" s="218" t="n">
+        <x:f>IF(SUMIF($B$6:$B$19,B15,$C$6:$C$19)=0,"n.a.",C15/SUMIF($B$6:$B$19,B15,$C$6:$C$19))</x:f>
         <x:v>0.1271585557299843</x:v>
       </x:c>
       <x:c r="E15" s="201" t="str">
@@ -3161,11 +3424,11 @@
       <x:c r="B16" s="201" t="str">
         <x:v>Outflow</x:v>
       </x:c>
-      <x:c r="C16" s="205" t="n">
+      <x:c r="C16" s="217" t="n">
         <x:v>6800</x:v>
       </x:c>
-      <x:c r="D16" s="206" t="n">
-        <x:f>C16/SUMIF($B$6:$B$19,B16,$C$6:$C$19)</x:f>
+      <x:c r="D16" s="218" t="n">
+        <x:f>IF(SUMIF($B$6:$B$19,B16,$C$6:$C$19)=0,"n.a.",C16/SUMIF($B$6:$B$19,B16,$C$6:$C$19))</x:f>
         <x:v>0.10675039246467818</x:v>
       </x:c>
       <x:c r="E16" s="201" t="str">
@@ -3179,11 +3442,11 @@
       <x:c r="B17" s="201" t="str">
         <x:v>Outflow</x:v>
       </x:c>
-      <x:c r="C17" s="205" t="n">
+      <x:c r="C17" s="217" t="n">
         <x:v>6200</x:v>
       </x:c>
-      <x:c r="D17" s="206" t="n">
-        <x:f>C17/SUMIF($B$6:$B$19,B17,$C$6:$C$19)</x:f>
+      <x:c r="D17" s="218" t="n">
+        <x:f>IF(SUMIF($B$6:$B$19,B17,$C$6:$C$19)=0,"n.a.",C17/SUMIF($B$6:$B$19,B17,$C$6:$C$19))</x:f>
         <x:v>0.09733124018838304</x:v>
       </x:c>
       <x:c r="E17" s="201" t="str">
@@ -3197,11 +3460,11 @@
       <x:c r="B18" s="201" t="str">
         <x:v>Outflow</x:v>
       </x:c>
-      <x:c r="C18" s="205" t="n">
+      <x:c r="C18" s="217" t="n">
         <x:v>3400</x:v>
       </x:c>
-      <x:c r="D18" s="206" t="n">
-        <x:f>C18/SUMIF($B$6:$B$19,B18,$C$6:$C$19)</x:f>
+      <x:c r="D18" s="218" t="n">
+        <x:f>IF(SUMIF($B$6:$B$19,B18,$C$6:$C$19)=0,"n.a.",C18/SUMIF($B$6:$B$19,B18,$C$6:$C$19))</x:f>
         <x:v>0.05337519623233909</x:v>
       </x:c>
       <x:c r="E18" s="201" t="str">
@@ -3215,11 +3478,11 @@
       <x:c r="B19" s="201" t="str">
         <x:v>Outflow</x:v>
       </x:c>
-      <x:c r="C19" s="205" t="n">
+      <x:c r="C19" s="217" t="n">
         <x:v>2000</x:v>
       </x:c>
-      <x:c r="D19" s="206" t="n">
-        <x:f>C19/SUMIF($B$6:$B$19,B19,$C$6:$C$19)</x:f>
+      <x:c r="D19" s="218" t="n">
+        <x:f>IF(SUMIF($B$6:$B$19,B19,$C$6:$C$19)=0,"n.a.",C19/SUMIF($B$6:$B$19,B19,$C$6:$C$19))</x:f>
         <x:v>0.03139717425431711</x:v>
       </x:c>
       <x:c r="E19" s="201" t="str">
@@ -3254,7 +3517,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37b33371f1ad4b94"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4dd9a5d4c6c94099"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3326,7 +3589,7 @@
       <x:c r="B6" s="201" t="str">
         <x:v>Average attendance</x:v>
       </x:c>
-      <x:c r="C6" s="207" t="n">
+      <x:c r="C6" s="219" t="n">
         <x:v>800</x:v>
       </x:c>
       <x:c r="D6" s="201" t="str">
@@ -3343,7 +3606,7 @@
       <x:c r="B7" s="201" t="str">
         <x:v>Ticket price</x:v>
       </x:c>
-      <x:c r="C7" s="207" t="n">
+      <x:c r="C7" s="219" t="n">
         <x:v>12</x:v>
       </x:c>
       <x:c r="D7" s="201" t="str">
@@ -3360,7 +3623,7 @@
       <x:c r="B8" s="201" t="str">
         <x:v>Base matches</x:v>
       </x:c>
-      <x:c r="C8" s="207" t="n">
+      <x:c r="C8" s="219" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="D8" s="201" t="str">
@@ -3377,7 +3640,7 @@
       <x:c r="B9" s="201" t="str">
         <x:v>Matches including playoffs</x:v>
       </x:c>
-      <x:c r="C9" s="207" t="n">
+      <x:c r="C9" s="219" t="n">
         <x:v>12</x:v>
       </x:c>
       <x:c r="D9" s="201" t="str">
@@ -3394,7 +3657,7 @@
       <x:c r="B10" s="201" t="str">
         <x:v>Average concession spend</x:v>
       </x:c>
-      <x:c r="C10" s="207" t="n">
+      <x:c r="C10" s="219" t="n">
         <x:v>8.5</x:v>
       </x:c>
       <x:c r="D10" s="201" t="str">
@@ -3411,7 +3674,7 @@
       <x:c r="B11" s="201" t="str">
         <x:v>Average attendance</x:v>
       </x:c>
-      <x:c r="C11" s="207" t="n">
+      <x:c r="C11" s="219" t="n">
         <x:v>800</x:v>
       </x:c>
       <x:c r="D11" s="201" t="str">
@@ -3428,7 +3691,7 @@
       <x:c r="B12" s="201" t="str">
         <x:v>Ticket price</x:v>
       </x:c>
-      <x:c r="C12" s="207" t="n">
+      <x:c r="C12" s="219" t="n">
         <x:v>12</x:v>
       </x:c>
       <x:c r="D12" s="201" t="str">
@@ -3445,7 +3708,7 @@
       <x:c r="B13" s="201" t="str">
         <x:v>Base matches</x:v>
       </x:c>
-      <x:c r="C13" s="207" t="n">
+      <x:c r="C13" s="219" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="D13" s="201" t="str">
@@ -3462,7 +3725,7 @@
       <x:c r="B14" s="201" t="str">
         <x:v>Matches including playoffs</x:v>
       </x:c>
-      <x:c r="C14" s="207" t="n">
+      <x:c r="C14" s="219" t="n">
         <x:v>12</x:v>
       </x:c>
       <x:c r="D14" s="201" t="str">
@@ -3479,7 +3742,7 @@
       <x:c r="B15" s="201" t="str">
         <x:v>Average concession spend</x:v>
       </x:c>
-      <x:c r="C15" s="207" t="n">
+      <x:c r="C15" s="219" t="n">
         <x:v>8.5</x:v>
       </x:c>
       <x:c r="D15" s="201" t="str">
@@ -3531,7 +3794,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89e83ca375c74a24"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd8c42e9f5674f76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3571,7 +3834,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>Generated 2026-10-12 • deterministic pipeline • Synthetic demonstration data</x:v>
+        <x:v>Source reference 2026-10-12 · refreshed for candidate 6.0 · synthetic controls</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>
@@ -3619,19 +3882,23 @@
       <x:c r="B6" s="208" t="n">
         <x:v>67500</x:v>
       </x:c>
-      <x:c r="C6" s="208" t="n">
+      <x:c r="C6" s="243" t="n">
+        <x:f>'Monthly Cash'!B18</x:f>
         <x:v>67500</x:v>
       </x:c>
       <x:c r="D6" s="208" t="n">
+        <x:f>C6-B6</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E6" s="209" t="str">
+        <x:f>IF(ABS(D6)&lt;0.005,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="F6" s="201" t="str">
         <x:v>Analytics owner</x:v>
       </x:c>
       <x:c r="G6" s="201" t="str">
+        <x:f>IF(E6="PASS","Cleared","Blocked")</x:f>
         <x:v>Cleared</x:v>
       </x:c>
     </x:row>
@@ -3642,19 +3909,23 @@
       <x:c r="B7" s="208" t="n">
         <x:v>67500</x:v>
       </x:c>
-      <x:c r="C7" s="208" t="n">
+      <x:c r="C7" s="243" t="n">
+        <x:f>SUMIF('Income &amp; Expense'!B6:B19,"Inflow",'Income &amp; Expense'!C6:C19)</x:f>
         <x:v>67500</x:v>
       </x:c>
       <x:c r="D7" s="208" t="n">
+        <x:f>C7-B7</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E7" s="209" t="str">
+        <x:f>IF(ABS(D7)&lt;0.005,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="F7" s="201" t="str">
         <x:v>Analytics owner</x:v>
       </x:c>
       <x:c r="G7" s="201" t="str">
+        <x:f>IF(E7="PASS","Cleared","Blocked")</x:f>
         <x:v>Cleared</x:v>
       </x:c>
     </x:row>
@@ -3665,19 +3936,23 @@
       <x:c r="B8" s="208" t="n">
         <x:v>63700</x:v>
       </x:c>
-      <x:c r="C8" s="208" t="n">
+      <x:c r="C8" s="243" t="n">
+        <x:f>'Monthly Cash'!C18</x:f>
         <x:v>63700</x:v>
       </x:c>
       <x:c r="D8" s="208" t="n">
+        <x:f>C8-B8</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E8" s="209" t="str">
+        <x:f>IF(ABS(D8)&lt;0.005,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="F8" s="201" t="str">
         <x:v>Analytics owner</x:v>
       </x:c>
       <x:c r="G8" s="201" t="str">
+        <x:f>IF(E8="PASS","Cleared","Blocked")</x:f>
         <x:v>Cleared</x:v>
       </x:c>
     </x:row>
@@ -3688,19 +3963,23 @@
       <x:c r="B9" s="208" t="n">
         <x:v>63700</x:v>
       </x:c>
-      <x:c r="C9" s="208" t="n">
+      <x:c r="C9" s="243" t="n">
+        <x:f>SUMIF('Income &amp; Expense'!B6:B19,"Outflow",'Income &amp; Expense'!C6:C19)</x:f>
         <x:v>63700</x:v>
       </x:c>
       <x:c r="D9" s="208" t="n">
+        <x:f>C9-B9</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E9" s="209" t="str">
+        <x:f>IF(ABS(D9)&lt;0.005,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="F9" s="201" t="str">
         <x:v>Analytics owner</x:v>
       </x:c>
       <x:c r="G9" s="201" t="str">
+        <x:f>IF(E9="PASS","Cleared","Blocked")</x:f>
         <x:v>Cleared</x:v>
       </x:c>
     </x:row>
@@ -3711,19 +3990,23 @@
       <x:c r="B10" s="208" t="n">
         <x:v>3800</x:v>
       </x:c>
-      <x:c r="C10" s="208" t="n">
+      <x:c r="C10" s="243" t="n">
+        <x:f>'Monthly Cash'!D18</x:f>
         <x:v>3800</x:v>
       </x:c>
       <x:c r="D10" s="208" t="n">
+        <x:f>C10-B10</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E10" s="209" t="str">
+        <x:f>IF(ABS(D10)&lt;0.005,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="F10" s="201" t="str">
         <x:v>Analytics owner</x:v>
       </x:c>
       <x:c r="G10" s="201" t="str">
+        <x:f>IF(E10="PASS","Cleared","Blocked")</x:f>
         <x:v>Cleared</x:v>
       </x:c>
     </x:row>
@@ -3734,19 +4017,23 @@
       <x:c r="B11" s="208" t="n">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C11" s="208" t="n">
+      <x:c r="C11" s="243" t="n">
+        <x:f>COUNTA('Monthly Cash'!A6:A17)</x:f>
         <x:v>12</x:v>
       </x:c>
       <x:c r="D11" s="208" t="n">
+        <x:f>C11-B11</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E11" s="209" t="str">
+        <x:f>IF(ABS(D11)&lt;0.005,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="F11" s="201" t="str">
         <x:v>Analytics owner</x:v>
       </x:c>
       <x:c r="G11" s="201" t="str">
+        <x:f>IF(E11="PASS","Cleared","Blocked")</x:f>
         <x:v>Cleared</x:v>
       </x:c>
     </x:row>
@@ -3757,19 +4044,23 @@
       <x:c r="B12" s="208" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C12" s="208" t="n">
+      <x:c r="C12" s="243" t="n">
+        <x:f>IF(COUNTIF('Operating Assumptions'!A6:A15,"Men's")&gt;0,1,0)+IF(COUNTIF('Operating Assumptions'!A6:A15,"Women's")&gt;0,1,0)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="D12" s="208" t="n">
+        <x:f>C12-B12</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="E12" s="209" t="str">
+        <x:f>IF(ABS(D12)&lt;0.005,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="F12" s="201" t="str">
         <x:v>Analytics owner</x:v>
       </x:c>
       <x:c r="G12" s="201" t="str">
+        <x:f>IF(E12="PASS","Cleared","Blocked")</x:f>
         <x:v>Cleared</x:v>
       </x:c>
     </x:row>
@@ -3850,9 +4141,29 @@
     <x:mergeCell ref="A1:G2"/>
     <x:mergeCell ref="A3:G3"/>
   </x:mergeCells>
+  <x:conditionalFormatting sqref="D6:D12">
+    <x:cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
+      <x:formula>0.004999</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
+      <x:formula>-0.004999</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="2" priority="3" operator="greaterThan">
+      <x:formula>0.004999</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="3" priority="4" operator="lessThan">
+      <x:formula>-0.004999</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="4" priority="5" operator="greaterThan">
+      <x:formula>0.004999</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="5" priority="6" operator="lessThan">
+      <x:formula>-0.004999</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd32c1dd5ea34c6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86dd48398dc64eba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4855,7 +5166,7 @@
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>Recruiter-ready evidence pack for the sanitized, read-only portfolio demonstration</x:v>
+        <x:v>Candidate 6.0 · source reference 2026-10-12 · prepared 2026-10-18, not published</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>
@@ -4936,7 +5247,7 @@
         <x:v>Monthly Cash</x:v>
       </x:c>
       <x:c r="B11" s="201" t="str">
-        <x:v>Formula-driven cash movement and cumulative position</x:v>
+        <x:v>Cash receipts/payments and cumulative net change, not balance</x:v>
       </x:c>
       <x:c r="C11" s="200"/>
       <x:c r="D11" s="200"/>
@@ -5023,7 +5334,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="51" t="str">
-        <x:v>No staff contacts, source payees, bank transactions, private filenames or interview attribution. This workbook is a portfolio artifact, not an audited financial statement or production planning source.</x:v>
+        <x:v>No staff contacts, source payees, bank transactions, private filenames or interview attribution. Formula recalculation and artifact rendering are checked with the bundled workbook engine; this does not establish a native Excel refresh. Power BI source checks are separate from Desktop rendering. Private operating records are not included.</x:v>
       </x:c>
       <x:c r="B19" s="52"/>
       <x:c r="C19" s="52"/>

</xml_diff>